<commit_message>
Nomi leggibili: materie con la denominazione ministeriale (display_name), classi mostrate come «1A» con l'indirizzo a parte
</commit_message>
<xml_diff>
--- a/webui/data/vicepreside_liceo90/files/01_materie.xlsx
+++ b/webui/data/vicepreside_liceo90/files/01_materie.xlsx
@@ -486,10 +486,9 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arte</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>Storia dell'arte</t>
+        </is>
+      </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
@@ -499,7 +498,6 @@
       <c r="F2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -509,10 +507,9 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ConversazioneFrancese</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Conversazione in lingua francese</t>
+        </is>
+      </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
@@ -522,7 +519,6 @@
       <c r="F3" t="n">
         <v>0</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -532,10 +528,9 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ConversazioneInglese</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Conversazione in lingua inglese</t>
+        </is>
+      </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
@@ -545,7 +540,6 @@
       <c r="F4" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -555,10 +549,9 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ConversazioneSpagnolo</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>Conversazione in lingua spagnola</t>
+        </is>
+      </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
@@ -568,7 +561,6 @@
       <c r="F5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -578,10 +570,9 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ConversazioneTedesco</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>Conversazione in lingua tedesca</t>
+        </is>
+      </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
@@ -591,7 +582,6 @@
       <c r="F6" t="n">
         <v>0</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -601,10 +591,9 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DirittoEconomia</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>Diritto ed economia</t>
+        </is>
+      </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
@@ -614,7 +603,6 @@
       <c r="F7" t="n">
         <v>0</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -624,10 +612,9 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DisegnoArte</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>Disegno e storia dell'arte</t>
+        </is>
+      </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
@@ -637,7 +624,6 @@
       <c r="F8" t="n">
         <v>0</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -650,7 +636,6 @@
           <t>Filosofia</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
@@ -660,7 +645,6 @@
       <c r="F9" t="n">
         <v>0</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -673,7 +657,6 @@
           <t>Fisica</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
         <v>0</v>
       </c>
@@ -683,7 +666,6 @@
       <c r="F10" t="n">
         <v>0</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -693,10 +675,9 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Geostoria</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>Storia e geografia</t>
+        </is>
+      </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
@@ -706,7 +687,6 @@
       <c r="F11" t="n">
         <v>0</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -716,10 +696,9 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Greco</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>Lingua e cultura greca</t>
+        </is>
+      </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
@@ -729,7 +708,6 @@
       <c r="F12" t="n">
         <v>0</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -742,7 +720,6 @@
           <t>Informatica</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
         <v>0</v>
       </c>
@@ -752,7 +729,6 @@
       <c r="F13" t="n">
         <v>0</v>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -762,10 +738,9 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Italiano</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>Lingua e letteratura italiana</t>
+        </is>
+      </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
@@ -775,7 +750,6 @@
       <c r="F14" t="n">
         <v>0</v>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -785,10 +759,9 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Latino</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>Lingua e cultura latina</t>
+        </is>
+      </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
@@ -798,7 +771,6 @@
       <c r="F15" t="n">
         <v>0</v>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -808,10 +780,9 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LinguaFrancese</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>Lingua e cultura francese</t>
+        </is>
+      </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
@@ -821,7 +792,6 @@
       <c r="F16" t="n">
         <v>0</v>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -831,10 +801,9 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LinguaInglese</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>Lingua e cultura inglese</t>
+        </is>
+      </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
@@ -844,7 +813,6 @@
       <c r="F17" t="n">
         <v>0</v>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -854,10 +822,9 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LinguaSpagnola</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>Lingua e cultura spagnola</t>
+        </is>
+      </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
@@ -867,7 +834,6 @@
       <c r="F18" t="n">
         <v>0</v>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -877,10 +843,9 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>LinguaTedesca</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>Lingua e cultura tedesca</t>
+        </is>
+      </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
@@ -890,7 +855,6 @@
       <c r="F19" t="n">
         <v>0</v>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -903,7 +867,6 @@
           <t>Matematica</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="n">
         <v>0</v>
       </c>
@@ -913,7 +876,6 @@
       <c r="F20" t="n">
         <v>0</v>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -923,10 +885,9 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Religione</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>Religione cattolica / Attività alternative</t>
+        </is>
+      </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
@@ -936,7 +897,6 @@
       <c r="F21" t="n">
         <v>0</v>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -946,7 +906,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Scienzemotorie</t>
+          <t>Scienze motorie e sportive</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -963,7 +923,6 @@
       <c r="F22" t="n">
         <v>0</v>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -973,10 +932,9 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Scienzenaturali</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>Scienze naturali</t>
+        </is>
+      </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
@@ -986,7 +944,6 @@
       <c r="F23" t="n">
         <v>0</v>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -996,10 +953,9 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Scienzeumane</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>Scienze umane</t>
+        </is>
+      </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
@@ -1009,7 +965,6 @@
       <c r="F24" t="n">
         <v>0</v>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1022,7 +977,6 @@
           <t>Storia</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="n">
         <v>0</v>
       </c>
@@ -1032,7 +986,6 @@
       <c r="F25" t="n">
         <v>0</v>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>